<commit_message>
Add block variations across multiple pages with screenshots
- Expanded block inventory from 27 to 38 screenshots
- Added new "Block Reuse Summary" sheet showing blocks used on multiple pages
- Captured blocks on: Business Fiber, Mobility Portfolio pages
- New screenshots: pricing-cards-fiber, features-grid-fiber, offer-cards-fiber,
  faq-accordion-fiber, lead-form-fiber, hero-portfolio-mobility, offer-cards-mobility,
  guarantee-mobility, and more
- Each block row now shows specific page URL where it appears
- Blocks documented across 5 page types: Homepage, Product, Portfolio, Industry, Customer Story

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/att-business-detailed-inventory.xlsx
+++ b/att-business-detailed-inventory.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="126">
   <si>
     <t>AT&amp;T Business - Detailed Page &amp; Asset Inventory</t>
   </si>
@@ -31,15 +31,24 @@
     <t>~150</t>
   </si>
   <si>
-    <t>Block Variations Documented:</t>
-  </si>
-  <si>
-    <t>27</t>
+    <t>Block Types Documented:</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Block Variations (with pages):</t>
+  </si>
+  <si>
+    <t>36</t>
   </si>
   <si>
     <t>Screenshot References:</t>
   </si>
   <si>
+    <t>38</t>
+  </si>
+  <si>
     <t>Category</t>
   </si>
   <si>
@@ -76,6 +85,12 @@
     <t>Product</t>
   </si>
   <si>
+    <t>Business Fiber Internet</t>
+  </si>
+  <si>
+    <t>/products/business-fiber-internet.html</t>
+  </si>
+  <si>
     <t>Dynamic Defense</t>
   </si>
   <si>
@@ -85,12 +100,6 @@
     <t>P2</t>
   </si>
   <si>
-    <t>Business Fiber</t>
-  </si>
-  <si>
-    <t>/products/business-fiber-internet.html</t>
-  </si>
-  <si>
     <t>Office@Hand</t>
   </si>
   <si>
@@ -280,7 +289,10 @@
     <t>Block Type</t>
   </si>
   <si>
-    <t>Source Page</t>
+    <t>Page Type</t>
+  </si>
+  <si>
+    <t>Page URL</t>
   </si>
   <si>
     <t>Screenshot</t>
@@ -337,6 +349,15 @@
     <t>Support Contact</t>
   </si>
   <si>
+    <t>Product Hero</t>
+  </si>
+  <si>
+    <t>Offer Cards Carousel</t>
+  </si>
+  <si>
+    <t>Portfolio Hero</t>
+  </si>
+  <si>
     <t>Industry Hero</t>
   </si>
   <si>
@@ -358,13 +379,13 @@
     <t>Contact CTA Banner</t>
   </si>
   <si>
-    <t>Lead Form Industry</t>
-  </si>
-  <si>
     <t>Article Video Hero</t>
   </si>
   <si>
     <t>Customer Story</t>
+  </si>
+  <si>
+    <t>/learn/customer-stories/portx.html</t>
   </si>
   <si>
     <t>Highlights/Stats</t>
@@ -445,7 +466,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -484,7 +505,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -523,7 +544,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -562,7 +583,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -601,7 +622,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -640,7 +661,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -679,7 +700,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -718,7 +739,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -757,7 +778,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -796,7 +817,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -835,7 +856,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -874,7 +895,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -913,7 +934,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -952,7 +973,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -991,7 +1012,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1030,7 +1051,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1069,7 +1090,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1108,7 +1129,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1147,7 +1168,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1186,7 +1207,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1225,7 +1246,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1264,7 +1285,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1303,7 +1324,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1342,7 +1363,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1381,7 +1402,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1420,7 +1441,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1459,7 +1480,7 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -1480,6 +1501,357 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Picture 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="Picture 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Picture 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="31" name="Picture 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Picture 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="33" name="Picture 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId33" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="34" name="Picture 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId34" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="35" name="Picture 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3619500" cy="1047750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="36" name="Picture 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1821,7 +2193,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1862,7 +2234,15 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1885,342 +2265,342 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
         <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" t="s">
         <v>27</v>
-      </c>
-      <c r="C7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
         <v>37</v>
       </c>
-      <c r="C11" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
-      </c>
       <c r="E11" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E12" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E13" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D14" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" t="s">
         <v>49</v>
       </c>
-      <c r="D15" t="s">
-        <v>46</v>
-      </c>
       <c r="E15" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" t="s">
         <v>50</v>
-      </c>
-      <c r="C16" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E17" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C18" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E18" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D19" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E19" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D20" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E20" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2242,86 +2622,86 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D4" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -2332,320 +2712,531 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="55" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="5" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="7" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="11" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="D12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="14" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>108</v>
+      </c>
+      <c r="B15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="22" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>103</v>
       </c>
-      <c r="B14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="15" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>104</v>
-      </c>
-      <c r="B15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="16" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>105</v>
-      </c>
-      <c r="B16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="17" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>106</v>
-      </c>
-      <c r="B17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="18" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>107</v>
-      </c>
-      <c r="B18" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="19" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>108</v>
-      </c>
-      <c r="B19" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="20" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>109</v>
-      </c>
-      <c r="B20" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="21" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>110</v>
-      </c>
-      <c r="B21" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="22" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>111</v>
-      </c>
-      <c r="B22" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="23" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>112</v>
-      </c>
       <c r="B23" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C23" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="D23" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>113</v>
       </c>
       <c r="B24" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C24" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="25" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="D24" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>112</v>
+      </c>
+      <c r="B25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>102</v>
+      </c>
+      <c r="B26" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>114</v>
       </c>
-      <c r="B25" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="26" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="B27" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" t="s">
+        <v>48</v>
+      </c>
+      <c r="D27" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="28" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>115</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B28" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" t="s">
+        <v>48</v>
+      </c>
+      <c r="D28" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="29" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>116</v>
       </c>
-      <c r="C26" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="27" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="B29" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>117</v>
       </c>
-      <c r="B27" t="s">
-        <v>116</v>
-      </c>
-      <c r="C27" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="28" ht="120" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="B30" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30" t="s">
+        <v>48</v>
+      </c>
+      <c r="D30" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="31" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>118</v>
       </c>
-      <c r="B28" t="s">
-        <v>116</v>
-      </c>
-      <c r="C28" t="s">
-        <v>91</v>
+      <c r="B31" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" t="s">
+        <v>48</v>
+      </c>
+      <c r="D31" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="32" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>119</v>
+      </c>
+      <c r="B32" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32" t="s">
+        <v>48</v>
+      </c>
+      <c r="D32" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="33" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>120</v>
+      </c>
+      <c r="B33" t="s">
+        <v>49</v>
+      </c>
+      <c r="C33" t="s">
+        <v>48</v>
+      </c>
+      <c r="D33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>103</v>
+      </c>
+      <c r="B34" t="s">
+        <v>49</v>
+      </c>
+      <c r="C34" t="s">
+        <v>48</v>
+      </c>
+      <c r="D34" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="35" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>121</v>
+      </c>
+      <c r="B35" t="s">
+        <v>122</v>
+      </c>
+      <c r="C35" t="s">
+        <v>123</v>
+      </c>
+      <c r="D35" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="36" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>124</v>
+      </c>
+      <c r="B36" t="s">
+        <v>122</v>
+      </c>
+      <c r="C36" t="s">
+        <v>123</v>
+      </c>
+      <c r="D36" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" ht="120" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>125</v>
+      </c>
+      <c r="B37" t="s">
+        <v>122</v>
+      </c>
+      <c r="C37" t="s">
+        <v>123</v>
+      </c>
+      <c r="D37" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>